<commit_message>
O'Reilly Evans #1: entrega final (Excel 6 hojas, markups Bluebeam, paso 11/12 resueltos, RESUMEN_MATERIALES, EVALUACION_INTERNA, SEGUIMIENTO) + skill v80u
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BLzQaGqFUvXc5j4BtA8MyA
</commit_message>
<xml_diff>
--- a/cache_proyectos/oreilly/FINAL_FOR_REVIEW_2026-10-31/Take-off/OReilly_Evans_Takeoff_FINAL.xlsx
+++ b/cache_proyectos/oreilly/FINAL_FOR_REVIEW_2026-10-31/Take-off/OReilly_Evans_Takeoff_FINAL.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="468">
   <si>
     <t xml:space="preserve">O'Reilly Auto Parts Store - 23rd Ave., Evans, CO #1   |   METAL FRAMING &amp; DRYWALL TAKEOFF</t>
   </si>
@@ -694,7 +694,7 @@
     <t xml:space="preserve">3-5/8" metal stud (LF of material)</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: S24-OFF 76.5 + S24-RR 102 + S24-RR104S 51 + S43-OFF-W 59.5 + S43-OFF-E 59.5 + S43-OFF-S 86.33 + S43-RR103-W 59.5 + S43-RR-S 147.17 + S41-B-V 60 + S41-B-H 36 + S41-C-V 48 + S41-C-H 36 + S42-H1 333.81 + S42-H2 116.76 + S42-V1 248.25 + S42-V2 97.85 + KICK-S42-H2 56.57 + KICK-S42-V1 98.99 + STRUT-S42-HDR 75.78 + ANGLED-STRUT-S42-HDR 64 + STUD-TIES-ENTRY 238.07 = 2,151.58 LF (per wall: field + jambs + nodes + cripples x height; plus listed elements) | By gauge (stud gauge of each wall, from its type / stud schedule): 33 mil (20 ga) - 362S162-33 1,618.17 LF; elements (gauge in their operation) 533.41 LF</t>
+    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: S24-OFF 76.5 + S24-RR 102 + S24-RR104S 51 + S43-OFF-W 59.5 + S43-OFF-E 59.5 + S43-OFF-S 86.33 + S43-RR103-W 59.5 + S43-RR-S 147.17 + S41-B-V 60 + S41-B-H 36 + S41-C-V 48 + S41-C-H 36 + S42-H1 333.81 + S42-H2 116.76 + S42-V1 248.25 + S42-V2 97.85 + KICK-S42-H2 56.57 + KICK-S42-V1 98.99 + STRUT-S42-HDR 75.78 + ANGLED-STRUT-S42-HDR 64 + STUD-TIES-ENTRY 238.07 + CJ-DOUBLE-STUDS 62.96 = 2,214.54 LF (per wall: field + jambs + nodes + cripples x height; plus listed elements) | By gauge (stud gauge of each wall, from its type / stud schedule): 33 mil (20 ga) - 362S162-33 1,618.17 LF; elements (gauge in their operation) 596.37 LF</t>
   </si>
   <si>
     <t xml:space="preserve">Bracing 1-1/2" C.R. channel @ 48" O.C.</t>
@@ -730,13 +730,13 @@
     <t xml:space="preserve">2x lumber 16 ft</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: BLK-S42-HDR-NAILERS 151.55 + BLK-RR-ACCESSORIES 38 + BLK-WATER-HEATER 4 + BLK-TOP-NAILERS-FRONT 101.34 = 294.89 LF</t>
+    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: BLK-S42-HDR-NAILERS 151.55 + BLK-RR-ACCESSORIES 38 + BLK-WATER-HEATER 4 + BLK-TOP-NAILERS-FRONT 101.34 + BLK-CMU-OPENINGS 56.67 = 351.56 LF</t>
   </si>
   <si>
     <t xml:space="preserve">5/8" gypsum board, Type X</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: S21-N 1,313.91 + S21-E1 663.19 + S21-E2 159.15 + S21-S 1,173.25 + S21-W1 151.17 + S21-W2 408.44 + S24-OFF 93.5 + S43-OFF-W 151.24 + S43-OFF-E 151.62 + S43-OFF-S 192.5 + S43-RR103-W 81.95 + S43-RR-S 145.5 + S41-B-V 26 + S41-B-H 15.76 + S41-C-V 20 + S41-C-H 15.76 + S42-H1 1,050.69 + S42-H2 365.08 + S42-V1 706.32 + S42-V2 231.2 + EXT-PIER-L-8 98.38 + EXT-PIER-R-8 98.38 + EXT-HEAD-8 155.27 + VEST-HD-C 42.62 + VEST-HD-B2 30.34 + VEST-HD-B1 30.34 + CLG-GWB-OFFICE-VEST 139.28 = 7,710.84 SF (faces: length x face height x layers - openings; ceilings: RCP area)</t>
+    <t xml:space="preserve">N/SHEET: not applicable (see note) | Breakdown [DERIVED]: S21-N 1,313.91 + S21-E1 663.19 + S21-E2 159.15 + S21-S 1,173.25 + S21-W1 151.17 + S21-W2 408.44 + S24-OFF 93.5 + S43-OFF-W 151.24 + S43-OFF-E 151.62 + S43-OFF-S 192.5 + S43-RR103-W 81.95 + S43-RR-S 145.5 + S41-B-V 26 + S41-B-H 15.76 + S41-C-V 20 + S41-C-H 15.76 + S42-H1 1,050.69 + S42-H2 365.08 + S42-V1 706.32 + S42-V2 231.2 + EXT-PIER-L-8 98.38 + EXT-PIER-R-8 98.38 + EXT-HEAD-8 155.27 + VEST-HD-C 42.62 + VEST-HD-B2 30.34 + VEST-HD-B1 30.34 + CLG-GWB-OFFICE-VEST 139.28 + GB-S42-HDR-UNDERSIDE 30.76 = 7,741.6 SF (faces: length x face height x layers - openings; ceilings: RCP area)</t>
   </si>
   <si>
     <t xml:space="preserve">5/8" gypsum board, Type X W.R. (water resistant)</t>
@@ -823,7 +823,7 @@
     <t xml:space="preserve">Drywall screws #7 x 1-1/4" Type S bugle head (board on 25/20 ga studs)</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: GA-216 | Inputs!B20 (Drywall screws per SF of board = 1.2) x 7957.66 SF of board</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: GA-216 | Inputs!B20 (Drywall screws per SF of board = 1.2) x 7988.42 SF of board</t>
   </si>
   <si>
     <t xml:space="preserve">Framing screws #8-18 x 1/2" pan head (25/20 ga studs)</t>
@@ -835,13 +835,13 @@
     <t xml:space="preserve">Power-driven fasteners, slab pins for the bottom track</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: slab pin spacing: see the operation (Inputs yield) | 226.82 LF of interior bottom track on slab / Inputs!B22 (Power-driven pin spacing (ft) = 1)</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: slab pin spacing: see the operation (Inputs yield) | 151.04 LF of interior bottom track on slab / Inputs!B22 (Power-driven pin spacing (ft) = 1)</t>
   </si>
   <si>
     <t xml:space="preserve">Expansion anchors Hilti 1/4" Kwik Bolt II, exterior bottom track @ 8" O.C.</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | 137.33 LF of exterior bottom track on slab / Inputs!B25 (Expansion anchor spacing (ft) = 0.6667)</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | 24 LF of exterior bottom track on slab / Inputs!B25 (Expansion anchor spacing (ft) = 0.6667)</t>
   </si>
   <si>
     <t xml:space="preserve">Joint compound, all purpose</t>
@@ -853,13 +853,13 @@
     <t xml:space="preserve">lb</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | Inputs!B23 (Joint compound (lb per SF) = 0.072) x 8412.97 SF of board</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | Inputs!B23 (Joint compound (lb per SF) = 0.072) x 8443.73 SF of board</t>
   </si>
   <si>
     <t xml:space="preserve">Joint tape, paper</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | Inputs!B24 (Joint tape (LF per SF) = 0.37) x 8412.97 SF of board</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: driver = the board / stud / bottom track rows of this sheet | Inputs!B24 (Joint tape (LF per SF) = 0.37) x 8443.73 SF of board</t>
   </si>
   <si>
     <t xml:space="preserve">Level 5 finish</t>
@@ -910,7 +910,7 @@
     <t xml:space="preserve">slab pins: pin spacing: carried one pin every 12.0" (Estimator criterion (Handoff - Approved: tightest of the three in the set, SILL TRACK ANCHORAGE interior @ 12" O.C.)); alternatives: one row @ 16" / one row @ 24"</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta 16in: -56.7 pcs; 24in: -113.41 pcs | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) Plans / specs: delta 16in: -37.76 pcs; 24in: -75.52 pcs | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-ACC-stud-reinforcement-mep</t>
@@ -928,7 +928,7 @@
     <t xml:space="preserve">Top of studs / Z-furring at the PEMB roof: bottom of purlin elevation not printed - where: S21-*, S42-H1, S42-H2, S42-V1, S42-V2, VEST-HD-* - carried: loaded to the top of purlin / eave elevation (conservative, rule 53.3)</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (2/A3.2, 1/A3.1, 3/S5.1): Studs and furring stop under the PEMB purlins / eave strut; T.O. eave 114'-7 1/2" (E) to 116'-4 3/4" (W) printed, purlin depth by P.E.M.B. shop drawings (A1.1 general note D) - delta minus purlin depth (~8" typical Z purlin) on every full-height stud, furring and board face: about -0.67 ft x LF of S21 (250.7 LF), S42 full (46.8 LF), heads | (B) Trade code (AISI S240-20 B1; ASTM C754 sec. 6): Code: no height rule; AISI S240 / ASTM C754 require the stud to bear on structure - height from shop drawings - delta same as A | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) Studs and furring stop under the PEMB purlins / eave strut; T.O. eave 114'-7 1/2" (E) to 116'-4 3/4" (W) printed, purlin depth by P.E.M.B. shop drawings (A1.1 general note D) | 2/A3.2, 1/A3.1, 3/S5.1 | delta minus purlin depth (~8" typical Z purlin) on every full-height stud, furring and board face: about -0.67 ft x LF of S21 (250.7 LF), S42 full (46.8 LF), heads | (B) Code: no height rule; AISI S240 / ASTM C754 require the stud to bear on structure - height from shop drawings | AISI S240-20 B1; ASTM C754 sec. 6 | delta same as A | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-02</t>
@@ -937,7 +937,7 @@
     <t xml:space="preserve">S24 Z-furring height and board on the CMU above the 8'-6" hard lid (office 102, R.R. 103/104) - where: S24-OFF, S24-RR, S24-RR104S - carried: S24 Z-furring loaded to the eave (14.625 / 14.71 ft) = 336.89 LF (misc item ZF-S24); board only to 8'-6" on the studs</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (S24/A1.1): S24/A1.1 draws 150ZF125-18 Z-furring + polyiso on the CMU behind the 8'-6" stud lining; height not stated (S21 goes to the roof per 3/A3.2) - delta + Z-furring 24" O.C. x 14.6 ft on 11.0 + 16.17 + 8.5 = 35.7 LF of CMU (about 19 pcs) and, if boarded above the hard lid, + 35.7 x 6.1 = 218 SF 5/8" Type X | (B) Trade code (IECC C402.1 (insulation continuity)): No code requirement for furring above a ceiling (energy code continuity of insulation only) - delta none | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) S24/A1.1 draws 150ZF125-18 Z-furring + polyiso on the CMU behind the 8'-6" stud lining; height not stated (S21 goes to the roof per 3/A3.2) | S24/A1.1 | delta + Z-furring 24" O.C. x 14.6 ft on 11.0 + 16.17 + 8.5 = 35.7 LF of CMU (about 19 pcs) and, if boarded above the hard lid, + 35.7 x 6.1 = 218 SF 5/8" Type X | (B) No code requirement for furring above a ceiling (energy code continuity of insulation only) | IECC C402.1 (insulation continuity) | delta none | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-03</t>
@@ -946,16 +946,16 @@
     <t xml:space="preserve">S42 header wall extension east of the S42 vertical wall - where: S42-H2 - carried: included (drawn on A1.1)</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.1, S4.1): A1.1 draws the header double line ~7.2 ft past the S42 corner (to the dimension line); S4.1 framing key plan ends the dashed header at the corner - delta -7.2 LF of header wall (S42-H2 25.44 -&gt; 18.27 ft) and its board / nailers | (B) Trade code (n/a): No code item - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) A1.1 draws the header double line ~7.2 ft past the S42 corner (to the dimension line); S4.1 framing key plan ends the dashed header at the corner | A1.1, S4.1 | delta -7.2 LF of header wall (S42-H2 25.44 -&gt; 18.27 ft) and its board / nailers | (B) No code item | n/a | delta n/a | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-04</t>
   </si>
   <si>
-    <t xml:space="preserve">South facade 36'-0" stucco band / windows D1-D2 drawn not to scale on A1.1 - where: EXT-SOUTH-BAND, S21-S openings - carried: 36'-0" printed taken</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.1, 4/A2.1, A5.2): A1.1 prints 36'-0" (drawn ~23.7 ft); 4/A2.1 elevation scales 36.0 ft; A5.2 D1/D2 11'-4 3/8" R.O. each - delta if the band were 23.7 ft: -12.3 LF of 6" studs x 7.97 ft and -98 SF sheathing | (B) Trade code (n/a): No code item - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">CLOSED (plan check): south facade 36'-0" stucco panel - the band measures 36.0 ft on A1.1, as printed - where: EXT-SOUTH-BAND, S21-S openings - carried: 36'-0" printed and measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) printed and measured agree | A1.1, A2.1 | delta 0 | (B) no code provision | n/a | delta 0 | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-05</t>
@@ -964,7 +964,7 @@
     <t xml:space="preserve">Hard-lid ceilings office/restrooms: board on top of the 600S162-54 joists - where: office 102, R.R. 103, R.R. 104 - carried: bottom (ceiling) board only</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (7/A4.2, A1.2): 7/A4.2 key 6 leaders reach the top of the joist box; schedule C-3 is the ceiling below - delta + 88 + 133.2 = 221.2 SF 5/8" Type X (WR in restrooms) if boarded on top | (B) Trade code (IBC 2021 703.2 (rated assemblies only)): Code: not required unless a rated assembly - delta none | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) 7/A4.2 key 6 leaders reach the top of the joist box; schedule C-3 is the ceiling below | 7/A4.2, A1.2 | delta + 88 + 133.2 = 221.2 SF 5/8" Type X (WR in restrooms) if boarded on top | (B) Code: not required unless a rated assembly | IBC 2021 703.2 (rated assemblies only) | delta none | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-06</t>
@@ -973,7 +973,7 @@
     <t xml:space="preserve">Entry pier / head interior finish and returns - where: EXT-PIER-*, EXT-HEAD-8 - carried: 5/8" Type X face loaded; RC and 1/4" not loaded (no family)</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (1/A3.1, 7/A3.2, 1/A5.2): 1/A3.1, 7/A3.2, 1/A5.2: 5/8" Type X over 1/4" gypsum board on 087F125-33 resilient channel @ 24" horiz.; pier side returns not dimensioned - delta + 1/4" gypsum about 349 SF and + 087F125-33 RC about 243 LF (piers 2 x 10 rows x 6.0 + head 4 rows x 30.67); returns + ~2 x 2 x 1.2 ft x 20.7 ft studs/sheathing | (B) Trade code (n/a): Code: no requirement - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) 1/A3.1, 7/A3.2, 1/A5.2: 5/8" Type X over 1/4" gypsum board on 087F125-33 resilient channel @ 24" horiz.; pier side returns not dimensioned | 1/A3.1, 7/A3.2, 1/A5.2 | delta + 1/4" gypsum about 349 SF and + 087F125-33 RC about 243 LF (piers 2 x 10 rows x 6.0 + head 4 rows x 30.67); returns + ~2 x 2 x 1.2 ft x 20.7 ft studs/sheathing; head underside (1/A5.2): +36 SF 5/8" X, +36 SF 1/4", +30.67 LF corner bead | (B) Code: no requirement | n/a | delta n/a | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-07</t>
@@ -982,7 +982,7 @@
     <t xml:space="preserve">Restroom wall finish W-4 sanitary wall and ceiling panel system - where: R.R. 103, R.R. 104 - carried: not loaded (finish trade); frp_none_reason</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.2): A1.2 schedule W-4 at R.R. 103/104 walls (MFG refer project manual) - delta + FRP-type panel on 4 walls of each restroom: about 2 x (2 x 7.83 + 2 x 8.5) x 8.5 = 555 SF if in the drywall scope | (B) Trade code (IBC 2021 1210.2.2): Code: smooth nonabsorbent surface to 4'-0" at urinals / water closets - delta finish to 4'-0" only: about 260 SF | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) A1.2 schedule W-4 at R.R. 103/104 walls (MFG refer project manual) | A1.2 | delta + FRP-type panel on 4 walls of each restroom: about 2 x (2 x 7.83 + 2 x 8.5) x 8.5 = 555 SF if in the drywall scope | (B) Code: smooth nonabsorbent surface to 4'-0" at urinals / water closets | IBC 2021 1210.2.2 | delta finish to 4'-0" only: about 260 SF | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-08</t>
@@ -991,7 +991,7 @@
     <t xml:space="preserve">MEP sweep excluded by the estimator (2026-10-31) - where: all stud walls - carried: 0 counted</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (SHEET_MAP (estimator exclusion)): MEP sheets not read: duct / pipe penetrations, framed openings and stud reinforcement not counted - delta per duct crossing a stud wall: + MAX(1, ROUNDUP(width/24")) plates and 1 sleeve | (B) Trade code (n/a): Code: n/a - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) MEP sheets not read: duct / pipe penetrations, framed openings and stud reinforcement not counted | SHEET_MAP (estimator exclusion) | delta per duct crossing a stud wall: + MAX(1, ROUNDUP(width/24")) plates and 1 sleeve | (B) Code: n/a | n/a | delta n/a | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-09</t>
@@ -1000,7 +1000,7 @@
     <t xml:space="preserve">S42 header wall bracing members not dimensioned (kicker length, angled strut length, 600S200-54 purlin members, track brace splices) - where: S42-H2, S42-V1 - carried: kickers 7.07 ft (45 deg), angled struts 8.0 ft; 600S200-54 not loaded</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (S5.1): 1/S5.1, 2/S5.1, 4/S5.1, 5/S5.1 give spacing only (kickers @ 48", angled strut @ 16'-0", 600S200-54 @ 24" / 48", 5'-0"+- reach) - delta kicker length +-1 ft each = +-22 LF; 600S200-54 pieces (not loaded): about ROUNDUP(L/2)+1 per header wall x purlin spacing (not printed) | (B) Trade code (AISI S240-20 B3.2): Code: AISI S240 bracing design by the specialty engineer - delta per engineer | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) 1/S5.1, 2/S5.1, 4/S5.1, 5/S5.1 give spacing only (kickers @ 48", angled strut @ 16'-0", 600S200-54 @ 24" / 48", 5'-0"+- reach) | S5.1 | delta kicker length +-1 ft each = +-22 LF; 600S200-54 pieces (not loaded): about ROUNDUP(L/2)+1 per header wall x purlin spacing (not printed); 2/S5.1: +16 L4x4x3/16 clip angles, +32 A307 bolts, +22 2x2x14 ga clips, +44 #10 SDS; #10 screws at kicker / strut / splice +400 | (B) Code: AISI S240 bracing design by the specialty engineer | AISI S240-20 B3.2 | delta per engineer | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-10</t>
@@ -1009,7 +1009,7 @@
     <t xml:space="preserve">Blocking quantities for toilet accessories, fire extinguishers, water heater, wall sign, 14/A4.1 key 12 - where: R.R. 103/104, S42, EXT-HEAD - carried: 48 LF loaded (accessories 38, extinguishers 6, water heater 4); 14/A4.1 key 12 and wall-sign backing not loaded</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A4.1, A4.2, A3.1): A4.1 accessory note 1, A4.1 key 17, A4.2 key 21, A3.1 key 31, 14/A4.1 key 12 call FRT blocking / backing without lengths - delta +-2 ft per accessory; 14/A4.1 key 12 continuous FRT 2x blocking along the Parts A walls would add up to ~140 LF (S42 Parts A faces) x rows | (B) Trade code (ICC A117.1-2017 609.8): Code: grab bars 250 lbf - delta as option A | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) A4.1 accessory note 1, A4.1 key 17, A4.2 key 21, A3.1 key 31, 14/A4.1 key 12 call FRT blocking / backing without lengths | A4.1, A4.2, A3.1 | delta +-2 ft per accessory; 14/A4.1 key 12 continuous FRT 2x blocking along the Parts A walls would add up to ~140 LF (S42 Parts A faces) x rows; plumbing fixture backing (C/A4.1) +12 LF | (B) Code: grab bars 250 lbf | ICC A117.1-2017 609.8 | delta as option A | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-11</t>
@@ -1018,7 +1018,7 @@
     <t xml:space="preserve">J molding / corner bead at gypsum perimeter transitions (A1.1 note 3.C) and the S42 header bottom - where: S42-H2, S42-V1, S21-* - carried: only 7/A4.2 corner bead and 2/A4.2 reveals loaded</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.1, 6/A4.2): A1.1 note 3.C J molding, reglets or corner bead at transitions to dissimilar materials; 6/A4.2 board wraps the header bottom - delta + corner bead 2 x 75.8 = 151.6 LF at the header bottoms; + J mold at board tops against the PEMB roof (S21/S42 tops ~ 330 LF) | (B) Trade code (ASTM C840-23 18.1): ASTM C840 sec. 18 trim at exposed edges - delta same | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) A1.1 note 3.C J molding, reglets or corner bead at transitions to dissimilar materials; 6/A4.2 board wraps the header bottom | A1.1, 6/A4.2 | delta + corner bead 2 x 75.8 = 151.6 LF at the header bottoms; + J mold at board tops against the PEMB roof (S21/S42 tops ~ 330 LF) | (B) ASTM C840 sec. 18 trim at exposed edges | ASTM C840-23 18.1 | delta same | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-12</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">Diagonal wall bracing 3" x 16 ga flat strap at corner faces of free standing partitions (A1.1 note 2.B) - where: S41-* - carried: not loaded</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.1 note 2.B): Which partitions are 'free standing' is not shown (S41 boxes, office/restroom boxes tied by joists, S42 braced per S5.1) - delta 2 straps x diagonal of each S41 leg face (~12.2 ft) x 4 legs = ~98 LF of 3" x 16 ga strap | (B) Trade code (AISI S240-20): AISI S240 bracing per design - delta per engineer | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) Which partitions are 'free standing' is not shown (S41 boxes, office/restroom boxes tied by joists, S42 braced per S5.1) | A1.1 note 2.B | delta 2 straps x diagonal of each S41 leg face (~12.2 ft) x 4 legs = ~98 LF of 3" x 16 ga strap | (B) AISI S240 bracing per design | AISI S240-20 | delta per engineer | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-13</t>
@@ -1036,16 +1036,25 @@
     <t xml:space="preserve">Metal headers at CMU openings (doors 2, 3, 7; windows D1, D2) in the Z-furring - where: S21-N, S21-S - carried: 0 (masonry lintels by mason)</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (S4.1, A5.1, A5.2): S4.1 masonry lintel schedule; 1/A5.1, 3/A5.1, 5/A5.1, 11/A5.2 show no metal header in the furring - delta if a 2-piece furring head were wanted: (R.O. + 1.333) x 2 per opening = 14.67 + 9.33 + 9.33 + 25.4 + 25.4 = 84.1 LF | (B) Trade code (n/a): Code: none - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) S4.1 masonry lintel schedule; 1/A5.1, 3/A5.1, 5/A5.1, 11/A5.2 show no metal header in the furring | S4.1, A5.1, A5.2 | delta if a 2-piece furring head were wanted: (R.O. + 1.333) x 2 per opening = 14.67 + 9.33 + 9.33 + 25.4 + 25.4 = 84.1 LF | (B) Code: none | n/a | delta n/a | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-14</t>
   </si>
   <si>
-    <t xml:space="preserve">Vestibule head walls / ceiling framing member and height - where: VEST-HD-*, JOISTS-VESTIBULE - carried: 600S162-43 heads to T.O. high eave 116'-4 1/4"; joists 600S162-43 @ 24"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (3/A3.1, 3/A5.2): 3/A3.1 key 8 600S162-43 @ 24" attached to PEMB; vestibule ceiling joists drawn under key 8; top at the purlin (not printed) - delta -0.67 ft on 20.6 LF of head if the purlin is 8" deep | (B) Trade code (n/a): AISI S240 - delta n/a | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">Vestibule head walls / ceiling framing member and height - where: VEST-HD-*, JOISTS-VESTIBULE - carried: vestibule heads carried 600S162-54 (16 ga, S4.1 key note 3 governs, A1.1 note 2.D) to the top of purlin; joists 600S162-43 @ 24" (3/A3.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) 3/A3.1 key 8 600S162-43 @ 24" attached to PEMB; vestibule ceiling joists drawn under key 8; top at the purlin (not printed) | 3/A3.1, 3/A5.2 | delta if 600S162-43 (3/A3.1 key 8): same LF, gauge 18 instead of 16 on 20.57 LF of heads; -0.67 ft x 20.6 LF if the purlin is 8" deep | (B) AISI S240 | n/a | delta n/a | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gypsum board finish level not printed (no project manual in the set; A1.1 notes silent) - where: all gypsum board - carried: Level 4 (joint compound + tape quantified), no Level 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) nothing printed (A1.1 notes 3.A-3.C; A1.2 W-2 semi-gloss paint) | A1.1, A1.2 | delta 0 | (B) Level 5 recommended under semi-gloss paint | GA-214 / ASTM C840 | delta + Level 5 SF = painted board SF | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-16</t>
@@ -1054,16 +1063,106 @@
     <t xml:space="preserve">Track at the top / bottom of the S21 Z-furring - where: S21 furring on the exterior CMU (6 walls) - carried: no track (none drawn on S21/A1.1 or the wall sections)</t>
   </si>
   <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (S21/A1.1): S21 type and 1/A3.2, 2/A3.2 draw the Z-furring on the CMU without track - delta 0 | (B) Trade code (ASTM C754 (furring attachment)): Furring J-track / runner at top and bottom if required by the installer - delta + 250.71 LF bottom + 250.71 LF top 1-1/2" track | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RFI-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gypsum board finish level not printed (no project manual in the set; A1.1 notes silent) - where: all gypsum board - carried: Level 4 (joint compound + tape quantified), no Level 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(A) Plans / specs: delta (A) Plans / specs (A1.1 interior wall &amp; ceiling notes 3.A-3.C; A1.2 finish W-2 semi-gloss paint): nothing printed - delta 0 | (B) Trade code (GA-214 / ASTM C840: semi-gloss paint finish is recommended at Level 5): Level 5 skim coat on painted walls - delta + Level 5 SF = painted board SF | (C) Other: ____ | (B) Trade code: no applicable code provision cited | (C) Other: ____</t>
+    <t xml:space="preserve">(A) S21 type and 1/A3.2, 2/A3.2 draw the Z-furring on the CMU without track | S21/A1.1 | delta 0 | (B) Furring J-track / runner at top and bottom if required by the installer | ASTM C754 (furring attachment) | delta + 250.71 LF bottom + 250.71 LF top 1-1/2" track | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRT 2x4 blocking at the window D1 / D2 openings in the CMU - where: south facade D1, D2 - carried: not loaded (window rough opening of D1 / D2 not dimensioned on A5.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) 11/A5.2 draws FRT 2x4 blocking anchored to masonry at the window head / jambs | 11/A5.2 | delta + (W + 2 x H) per window, about +2 x 34 LF; FRT plywood at the D1 / D2 heads (11/A5.2) +15 SF | (B) no code provision | n/a | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gypsum board control joints on the S21 furring (walls over 30 ft and at masonry control joints) - where: S21-N, S21-E1, S21-S - carried: not loaded: joint locations follow the masonry control joints of the exterior elevations, not dimensioned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) A1.1 note 3.A: control joints in partition lengths over 30 ft and at masonry control joints | 3.A/A1.1, A2.1 key 23 | delta about +77 LF of control joint (Step 12 estimate) | (B) control joints at 30 ft max | ASTM C840 / GA-216 | delta + 1 joint per 30 ft of S21 run x height | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moisture resistant Type X at the janitor sink area (A1.1 note 3.B) - where: mop sink area, 13/A4.1 - carried: regular Type X carried outside the restrooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) W.R. at janitor sink areas: extent not dimensioned | 3.B/A1.1, 13/A4.1 | delta reclass +43 to +241 SF from Type X to Type X W.R. (no net SF change) | (B) MR board behind wet fixtures | GA-216 | delta same reclass | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simpson FCB43.5 clips and their fasteners at the exterior stud connections (S5.2 key notes 16 / 23, 1/S5.3, 3/S5.3) - where: entry piers, head wall - carried: not loaded: clip count per connection not dimensioned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) clips per stud at the CMU / wind beam connection | 1/S5.3, 3/S5.3 | delta +146 FCB43.5 clips, +584 #12-14 screws, +168 Tapcon, +124 #12-24 (Step 12 count) | (B) per manufacturer | Simpson catalog | delta same | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sheathing screws #6 x 1-1/4" corrosion resistant (S5.2 key 8) vs #10 (S1.1 7.D) - where: glass mat / FRT plywood sheathing - carried: not loaded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) sheathing screws at the printed spacing | S5.2, S1.1 | delta about +1,075 screws | (B) #10 screws per S1.1 7.D | S1.1 7.D | delta same count, #10 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRT 2x nailers on the CMU parapet (5-6/A3.2, 4-5/A3.4, 2/A6.1) and 1/2" anchors - where: CMU parapets - carried: EXCLUDED: wood nailers anchored to the masonry parapet are rough carpentry / roofing (Div 06), not framing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) if carried by the framing sub | 5/A3.2, 2/A6.1 | delta +544 to 816 LF FRT 2x + 1/2" anchors | (B) n/a | n/a | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRT 2x nailers inside the concealed PEMB column enclosures (1/A4.2 key 10) - where: key note 1 columns, A1.1 - carried: not loaded: enclosure by others (1/A4.2 key 16); column count not in our scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) nailers per concealed column | 1/A4.2 | delta about +48 LF per column | (B) n/a | n/a | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security shutters 'may be required' (H/A5.2) - where: storefront A - carried: not loaded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) framing for shutter housing if required | H/A5.2 | delta 0 now; header / box framing if the shutter is added | (B) n/a | n/a | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deflection track product: 3" x 14 ga deep-leg slotted track (3/S5.1, 4/S5.1) vs track at stud gauge - where: S42 full-height walls, S21 / S24 tops - carried: LF carried in the top / deflection track rows at stud gauge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) deep-leg 14 ga slotted track at walls to the purlin | 3/S5.1, 4/S5.1 | delta same LF, product upgrade on the full-height S42 walls (46.84 LF) | (B) deflection per A1.1 note 2.C | A1.1 2.C | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interior bottom track anchors: Titen HD @ 48" (3/S5.1, 4/S5.1, S1.1 7.F/G) vs slab pins - where: interior walls on slab - carried: slab pins carried (151.04 pcs, Inputs spacing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) Titen HD @ 48" printed for the S42 floor walls | 3/S5.1, S1.1 | delta -151.04 pins, + about 69 Titen HD (Step 12 count) | (B) n/a | n/a | delta 0 | (C) Other: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stud-to-track screws #10 (S1.1 7.E) vs #8 carried; framing screws charged on the Z-furring - where: all framing - carried: #8-18 x 1/2" carried by the tool rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) #10 screws printed | S1.1 | delta same count, #10 instead of #8; -668 screws on the Z-furring (no track) | (B) n/a | n/a | delta 0 | (C) Other: ____</t>
   </si>
   <si>
     <t xml:space="preserve">0 questions in total, asked ONE at a time in this order: floor plan (partition types A-Z), then the details the floor plan calls, in order</t>
@@ -1330,7 +1429,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "3f08a25190440ff312894c385c03cb32cfa4fd64d3dd5b6d2a18f1613025af81", "evidencias": "a733add1c3f7df82ebc21662de53a041d63c1ea8dedf2ec71dee7c6ac9902895", "familias_out": "40c51f2aa05bbc6f4abbeb3015bfcd5b885e4e7e556cc9787de44edd128a9fd4", "reglas": "ef90708f6b29fb8f4183862452477e382e4b0b487de236ebf5bd2eb12c76a0f8", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "a1027b13b49f3390f1da69d595cd0413455c70f9b890e9e803616cf6497665ce", "evidencias": "049573fa2d17514c730615e6fbddf8604988953fd9bc7e79bd0720f6d13c30e7", "familias_out": "e1f706d7ad4696e96a2350ea6f2a92e43c13ddc263b270f80367c8c65a681174", "reglas": "416b0052865ced4ef0056681dee972ee1f64972ce9e9e9d6b84a5bdb739dd0c5", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -3669,7 +3768,7 @@
         <v>200</v>
       </c>
       <c r="C15" s="0" t="n">
-        <v>2151.58</v>
+        <v>2214.54</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -3677,18 +3776,18 @@
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">C15*D15</f>
-        <v>322.737</v>
+        <v>332.181</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">C15+E15</f>
-        <v>2474.317</v>
+        <v>2546.721</v>
       </c>
       <c r="G15" s="0" t="s">
         <v>217</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">ROUNDUP(F15/Inputs!$B$10,0)</f>
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="I15" s="0" t="s">
         <v>222</v>
@@ -3801,7 +3900,7 @@
         <v>200</v>
       </c>
       <c r="C19" s="0" t="n">
-        <v>294.89</v>
+        <v>351.56</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">Inputs!$B$6</f>
@@ -3809,18 +3908,18 @@
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">C19*D19</f>
-        <v>17.6934</v>
+        <v>21.0936</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">C19+E19</f>
-        <v>312.5834</v>
+        <v>372.6536</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>233</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">ROUNDUP(F19/Inputs!$B$26,0)</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I19" s="0" t="s">
         <v>234</v>
@@ -3834,7 +3933,7 @@
         <v>229</v>
       </c>
       <c r="C20" s="0" t="n">
-        <v>7710.82</v>
+        <v>7741.58</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">Inputs!$B$6</f>
@@ -3842,11 +3941,11 @@
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">C20*D20</f>
-        <v>462.6492</v>
+        <v>464.4948</v>
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">C20+E20</f>
-        <v>8173.4692</v>
+        <v>8206.0748</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>230</v>
@@ -4260,7 +4359,7 @@
         <v>249</v>
       </c>
       <c r="C33" s="0" t="n">
-        <v>9549.19</v>
+        <v>9586.1</v>
       </c>
       <c r="D33" s="0" t="n">
         <v>0</v>
@@ -4271,21 +4370,21 @@
       </c>
       <c r="F33" s="0" t="n">
         <f aca="false">C33+E33</f>
-        <v>9549.19</v>
+        <v>9586.1</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>250</v>
       </c>
       <c r="H33" s="0" t="n">
         <f aca="false">ROUNDUP(F33,0)</f>
-        <v>9550</v>
+        <v>9587</v>
       </c>
       <c r="I33" s="0" t="s">
         <v>265</v>
       </c>
       <c r="J33" s="0" t="n">
-        <f aca="false">Inputs!$B$20*7957.66</f>
-        <v>9549.192</v>
+        <f aca="false">Inputs!$B$20*7988.42</f>
+        <v>9586.104</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4332,7 +4431,7 @@
         <v>249</v>
       </c>
       <c r="C35" s="0" t="n">
-        <v>226.82</v>
+        <v>151.04</v>
       </c>
       <c r="D35" s="0" t="n">
         <v>0</v>
@@ -4343,21 +4442,21 @@
       </c>
       <c r="F35" s="0" t="n">
         <f aca="false">C35+E35</f>
-        <v>226.82</v>
+        <v>151.04</v>
       </c>
       <c r="G35" s="0" t="s">
         <v>250</v>
       </c>
       <c r="H35" s="0" t="n">
         <f aca="false">ROUNDUP(F35,0)</f>
-        <v>227</v>
+        <v>152</v>
       </c>
       <c r="I35" s="0" t="s">
         <v>269</v>
       </c>
       <c r="J35" s="0" t="n">
-        <f aca="false">226.82/Inputs!$B$22</f>
-        <v>226.82</v>
+        <f aca="false">151.04/Inputs!$B$22</f>
+        <v>151.04</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4368,7 +4467,7 @@
         <v>249</v>
       </c>
       <c r="C36" s="0" t="n">
-        <v>206</v>
+        <v>36</v>
       </c>
       <c r="D36" s="0" t="n">
         <v>0</v>
@@ -4379,21 +4478,21 @@
       </c>
       <c r="F36" s="0" t="n">
         <f aca="false">C36+E36</f>
-        <v>206</v>
+        <v>36</v>
       </c>
       <c r="G36" s="0" t="s">
         <v>250</v>
       </c>
       <c r="H36" s="0" t="n">
         <f aca="false">ROUNDUP(F36,0)</f>
-        <v>206</v>
+        <v>36</v>
       </c>
       <c r="I36" s="0" t="s">
         <v>271</v>
       </c>
       <c r="J36" s="0" t="n">
-        <f aca="false">137.33/Inputs!$B$25</f>
-        <v>205.984700764962</v>
+        <f aca="false">24/Inputs!$B$25</f>
+        <v>35.9982000899955</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4404,7 +4503,7 @@
         <v>273</v>
       </c>
       <c r="C37" s="0" t="n">
-        <v>605.73</v>
+        <v>607.95</v>
       </c>
       <c r="D37" s="0" t="n">
         <v>0</v>
@@ -4415,21 +4514,21 @@
       </c>
       <c r="F37" s="0" t="n">
         <f aca="false">C37+E37</f>
-        <v>605.73</v>
+        <v>607.95</v>
       </c>
       <c r="G37" s="0" t="s">
         <v>274</v>
       </c>
       <c r="H37" s="0" t="n">
         <f aca="false">ROUNDUP(F37,0)</f>
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="I37" s="0" t="s">
         <v>275</v>
       </c>
       <c r="J37" s="0" t="n">
-        <f aca="false">Inputs!$B$23*8412.97</f>
-        <v>605.73384</v>
+        <f aca="false">Inputs!$B$23*8443.73</f>
+        <v>607.94856</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4440,7 +4539,7 @@
         <v>200</v>
       </c>
       <c r="C38" s="0" t="n">
-        <v>3112.8</v>
+        <v>3124.18</v>
       </c>
       <c r="D38" s="0" t="n">
         <v>0</v>
@@ -4451,21 +4550,21 @@
       </c>
       <c r="F38" s="0" t="n">
         <f aca="false">C38+E38</f>
-        <v>3112.8</v>
+        <v>3124.18</v>
       </c>
       <c r="G38" s="0" t="s">
         <v>200</v>
       </c>
       <c r="H38" s="0" t="n">
         <f aca="false">ROUNDUP(F38,0)</f>
-        <v>3113</v>
+        <v>3125</v>
       </c>
       <c r="I38" s="0" t="s">
         <v>277</v>
       </c>
       <c r="J38" s="0" t="n">
-        <f aca="false">Inputs!$B$24*8412.97</f>
-        <v>3112.7989</v>
+        <f aca="false">Inputs!$B$24*8443.73</f>
+        <v>3124.1801</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4613,7 +4712,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -4838,6 +4937,127 @@
       </c>
       <c r="C20" s="0" t="s">
         <v>345</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>346</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>347</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>349</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>350</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>352</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>353</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>355</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>356</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>358</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>359</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>361</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>362</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>364</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>365</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>367</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>368</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>370</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>371</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>373</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>374</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>376</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>378</v>
       </c>
     </row>
   </sheetData>
@@ -4869,27 +5089,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>346</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>348</v>
+        <v>381</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>349</v>
+        <v>382</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>350</v>
+        <v>383</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>352</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -4919,366 +5139,366 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>353</v>
+        <v>386</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>354</v>
+        <v>387</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>355</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>357</v>
+        <v>390</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>359</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>360</v>
+        <v>393</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>361</v>
+        <v>394</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>362</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>363</v>
+        <v>396</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>364</v>
+        <v>397</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>366</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>367</v>
+        <v>400</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>368</v>
+        <v>401</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>369</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>370</v>
+        <v>403</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>371</v>
+        <v>404</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>372</v>
+        <v>405</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>373</v>
+        <v>406</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>374</v>
+        <v>407</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>375</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>376</v>
+        <v>409</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>377</v>
+        <v>410</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>378</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>379</v>
+        <v>412</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>380</v>
+        <v>413</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>381</v>
+        <v>414</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>382</v>
+        <v>415</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>383</v>
+        <v>416</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>384</v>
+        <v>417</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>385</v>
+        <v>418</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>386</v>
+        <v>419</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>387</v>
+        <v>420</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>388</v>
+        <v>421</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>389</v>
+        <v>422</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>390</v>
+        <v>423</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>391</v>
+        <v>424</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>392</v>
+        <v>425</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>393</v>
+        <v>426</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>394</v>
+        <v>427</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>395</v>
+        <v>428</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>396</v>
+        <v>429</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>397</v>
+        <v>430</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>431</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>398</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>365</v>
-      </c>
       <c r="D15" s="0" t="s">
-        <v>399</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>400</v>
+        <v>433</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>401</v>
+        <v>434</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>402</v>
+        <v>435</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>403</v>
+        <v>436</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>404</v>
+        <v>437</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>405</v>
+        <v>438</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>406</v>
+        <v>439</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>407</v>
+        <v>440</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>286</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>408</v>
+        <v>441</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>409</v>
+        <v>442</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>410</v>
+        <v>443</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>358</v>
+        <v>391</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>411</v>
+        <v>444</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>412</v>
+        <v>445</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>413</v>
+        <v>446</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>414</v>
+        <v>447</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>415</v>
+        <v>448</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>416</v>
+        <v>449</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>286</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>417</v>
+        <v>450</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>418</v>
+        <v>451</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>419</v>
+        <v>452</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>420</v>
+        <v>453</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>421</v>
+        <v>454</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>422</v>
+        <v>455</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>423</v>
+        <v>456</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>424</v>
+        <v>457</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>425</v>
+        <v>458</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>426</v>
+        <v>459</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>427</v>
+        <v>460</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>428</v>
+        <v>461</v>
       </c>
       <c r="C25" s="0" t="s">
         <v>286</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>429</v>
+        <v>462</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>430</v>
+        <v>463</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>431</v>
+        <v>464</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>432</v>
+        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -5302,12 +5522,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>433</v>
+        <v>466</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>